<commit_message>
Live Gemini evaluation (gemini-3.5-flash-lite); update default model; regenerate sample output with Gemini explanations
</commit_message>
<xml_diff>
--- a/sample_output/audit_report.xlsx
+++ b/sample_output/audit_report.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="330">
   <si>
     <t>metric</t>
   </si>
@@ -91,13 +91,13 @@
     <t>auto_approved</t>
   </si>
   <si>
-    <t>20261020T204005Z-db41c2</t>
-  </si>
-  <si>
-    <t>2026-10-20T20:40:05+00:00</t>
-  </si>
-  <si>
-    <t>mock</t>
+    <t>20261020T205936Z-a512ec</t>
+  </si>
+  <si>
+    <t>2026-10-20T20:59:36+00:00</t>
+  </si>
+  <si>
+    <t>gemini:gemini-3.5-flash-lite</t>
   </si>
   <si>
     <t>9460928031e3</t>
@@ -460,43 +460,40 @@
     <t>Procurement_Policy_2026.pdf p.1 Rule 10; Procurement_Policy_2026.pdf p.1 Rule 2</t>
   </si>
   <si>
-    <t>FLAG Q-003: Quoted USD 714.92 vs policy-expected USD 594.92 (variance +120.00, overquote; tolerance 0.01, Rule 8). Rate C-14 (2026-01-01..2026-12-31) applies for quote date 2026-09-18 (Rule 1). Also noted: UNEXPLAINED_VARIANCE. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-005: Quoted USD 394.83 vs policy-expected USD 309.83 (variance +85.00, overquote; tolerance 0.01, Rule 8). Rate B-14 (2026-01-01..2026-12-31) applies for quote date 2026-10-12 (Rule 1). Also noted: UNEXPLAINED_VARIANCE, NOTE_VENDOR_MISMATCH, UNAUTHORIZED_SURCHARGE. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-007: Quoted USD 798.90 vs policy-expected USD 728.90 (variance +70.00, overquote; tolerance 0.01, Rule 8). Rate A-NEW14 (2026-10-01..2026-12-31) applies for quote date 2026-10-12 (Rule 1). Also noted: UNEXPLAINED_VARIANCE, NOTE_VENDOR_MISMATCH, PROMPT_INJECTION_DETECTED. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-002: Quoted USD 604.44 vs policy-expected USD 544.47 (variance +59.97, overquote; tolerance 0.01, Rule 8). Rate B-14 (2026-01-01..2026-12-31) applies for quote date 2026-09-18 (Rule 1). Hypothesis: Rhodium finish charged although PO finish is Standard; settings counted as 4 instead of 2 (per earring instead of per pair). Also noted: FINISH_NOT_ON_PO, SETTING_COUNT_MISMATCH. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-012: Quoted USD 593.56 vs policy-expected USD 543.56 (variance +50.00, overquote; tolerance 0.01, Rule 8). Rate C-14 (2026-01-01..2026-12-31) applies for quote date 2026-10-21 (Rule 1). Also noted: UNEXPLAINED_VARIANCE. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-006: Quoted USD 1110.00 vs policy-expected USD 1070.00 (variance +40.00, overquote; tolerance 0.01, Rule 8). Rate C-18 (2026-01-01..2026-12-31) applies for quote date 2026-10-12 (Rule 1). Also noted: MISSING_SKU, UNEXPLAINED_VARIANCE, NOTE_VENDOR_MISMATCH, DUPLICATE_NOTICE, HISTORY_UNMAPPED. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-011: Quoted USD 716.80 vs policy-expected USD 681.80 (variance +35.00, overquote; tolerance 0.01, Rule 8). Rate B-18 (2026-01-01..2026-12-31) applies for quote date 2026-10-21 (Rule 1). Also noted: UNEXPLAINED_VARIANCE. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-009: Quoted USD 510.72 vs policy-expected USD 530.72 (variance -20.00, underquote; tolerance 0.01, Rule 8). Rate C-14 (2026-01-01..2026-12-31) applies for quote date 2026-10-21 (Rule 1). Also noted: UNEXPLAINED_VARIANCE. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>FLAG Q-010: Quoted USD 241.16 vs policy-expected USD 226.16 (variance +15.00, overquote; tolerance 0.01, Rule 8). Rate A-NEW14 (2026-10-01..2026-12-31) applies for quote date 2026-10-21 (Rule 1). Hypothesis: Rhodium finish charged although PO finish is Standard. Also noted: MISSING_SKU, FINISH_NOT_ON_PO. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>WITHIN_TOLERANCE Q-001: Quoted USD 409.32 vs policy-expected USD 409.32 (variance +0.00, exact match; tolerance 0.01, Rule 8). Rate A-OLD (2026-01-01..2026-09-30) applies for quote date 2026-09-18 (Rule 1). Also noted: RATE_CHANGE_NOTICE_IGNORED. No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>WITHIN_TOLERANCE Q-004: Quoted USD 687.96 vs policy-expected USD 687.96 (variance +0.00, exact match; tolerance 0.01, Rule 8). Rate A-OLD18 (2026-01-01..2026-09-30) applies for quote date 2026-09-18 (Rule 1). No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>WITHIN_TOLERANCE Q-008: Quoted USD 845.84 vs policy-expected USD 845.84 (variance +0.00, exact match; tolerance 0.01, Rule 8). Rate B-18 (2026-01-01..2026-12-31) applies for quote date 2026-10-12 (Rule 1). No automatic approval; a human reviewer decision is required (Rule 10).</t>
-  </si>
-  <si>
-    <t>template (mock provider)</t>
+    <t>For quote Q-003 with rate C-14 (2026-01-01..2026-12-31), the absolute variance of USD 120.00 exceeds the tolerance of 0.01 under Rule 8. No single pricing error reproduces the quoted total, indicating a possible undisclosed charge. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-005 with rate B-14 (2026-01-01..2026-12-31), the absolute variance of USD 85.00 exceeds the tolerance of 0.01 under Rule 8. An unauthorized surcharge of USD 75 was claimed without a signed exception. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-007 with rate A-NEW14 (2026-10-01..2026-12-31), the absolute variance of USD 70.00 exceeds the tolerance of 0.01 under Rule 8. Embedded instructions in the associated notice were quarantined and ignored. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-002 with rate B-14 (2026-01-01..2026-12-31), the absolute variance of USD 59.97 exceeds the tolerance of 0.01 under Rule 8. As a hypothesis, a rhodium finish was charged although the PO finish is standard violating Rule 6, and settings were counted as 4 instead of 2 violating Rule 3 and Rule 4. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-012 with rate C-14 (2026-01-01..2026-12-31), the absolute variance of USD 50.00 exceeds the tolerance of 0.01 under Rule 8 with an unexplained variance. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-006 with rate C-18 (2026-01-01..2026-12-31), the absolute variance of USD 40.00 exceeds the tolerance of 0.01 under Rule 8. The supplier did not provide a SKU. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-011 with rate B-18 (2026-01-01..2026-12-31), the absolute variance of USD 35.00 exceeds the tolerance of 0.01 under Rule 8 with an unexplained variance. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-009 with rate C-14 (2026-01-01..2026-12-31), the absolute variance of USD 20.00 exceeds the tolerance of 0.01. Underquotes must be identified and not automatically rejected pursuant to Rule 8. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-010 with rate A-NEW14 (2026-10-01..2026-12-31), the absolute variance of USD 15.00 exceeds the tolerance of 0.01 under Rule 8. As a hypothesis, a rhodium finish was charged although the PO finish is standard, violating Rule 6. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-001 with rate A-OLD (2026-01-01..2026-09-30), the quote date governs applicability under Rule 1. The variance is within tolerance. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-004 with rate A-OLD18 (2026-01-01..2026-09-30), the quote date governs under Rule 1 and the variance is within tolerance. A human reviewer decision is required.</t>
+  </si>
+  <si>
+    <t>For quote Q-008 with rate B-18 (2026-01-01..2026-12-31), the variance is within tolerance and expected costs match correctly. A human reviewer decision is required.</t>
   </si>
   <si>
     <t>pending</t>
@@ -1717,10 +1714,10 @@
         <v>146</v>
       </c>
       <c r="AA2" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB2" t="s">
         <v>158</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>159</v>
       </c>
       <c r="AG2" t="b">
         <v>0</v>
@@ -1803,10 +1800,10 @@
         <v>147</v>
       </c>
       <c r="AA3" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB3" t="s">
         <v>158</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>159</v>
       </c>
       <c r="AG3" t="b">
         <v>0</v>
@@ -1889,10 +1886,10 @@
         <v>148</v>
       </c>
       <c r="AA4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB4" t="s">
         <v>158</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>159</v>
       </c>
       <c r="AG4" t="b">
         <v>0</v>
@@ -1978,10 +1975,10 @@
         <v>149</v>
       </c>
       <c r="AA5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB5" t="s">
         <v>158</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>159</v>
       </c>
       <c r="AG5" t="b">
         <v>0</v>
@@ -2064,10 +2061,10 @@
         <v>150</v>
       </c>
       <c r="AA6" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB6" t="s">
         <v>158</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>159</v>
       </c>
       <c r="AG6" t="b">
         <v>0</v>
@@ -2120,7 +2117,7 @@
         <v>124</v>
       </c>
       <c r="P7">
-        <v>0.742</v>
+        <v>0.792</v>
       </c>
       <c r="Q7">
         <v>366</v>
@@ -2150,10 +2147,10 @@
         <v>151</v>
       </c>
       <c r="AA7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB7" t="s">
         <v>158</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>159</v>
       </c>
       <c r="AG7" t="b">
         <v>0</v>
@@ -2236,10 +2233,10 @@
         <v>152</v>
       </c>
       <c r="AA8" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB8" t="s">
         <v>158</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>159</v>
       </c>
       <c r="AG8" t="b">
         <v>0</v>
@@ -2322,10 +2319,10 @@
         <v>153</v>
       </c>
       <c r="AA9" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB9" t="s">
         <v>158</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>159</v>
       </c>
       <c r="AG9" t="b">
         <v>0</v>
@@ -2378,7 +2375,7 @@
         <v>124</v>
       </c>
       <c r="P10">
-        <v>0.775</v>
+        <v>0.8</v>
       </c>
       <c r="Q10">
         <v>159.6</v>
@@ -2411,10 +2408,10 @@
         <v>154</v>
       </c>
       <c r="AA10" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB10" t="s">
         <v>158</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>159</v>
       </c>
       <c r="AG10" t="b">
         <v>0</v>
@@ -2497,10 +2494,10 @@
         <v>155</v>
       </c>
       <c r="AA11" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB11" t="s">
         <v>158</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>159</v>
       </c>
       <c r="AG11" t="b">
         <v>0</v>
@@ -2583,10 +2580,10 @@
         <v>156</v>
       </c>
       <c r="AA12" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB12" t="s">
         <v>158</v>
-      </c>
-      <c r="AB12" t="s">
-        <v>159</v>
       </c>
       <c r="AG12" t="b">
         <v>0</v>
@@ -2669,10 +2666,10 @@
         <v>157</v>
       </c>
       <c r="AA13" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB13" t="s">
         <v>158</v>
-      </c>
-      <c r="AB13" t="s">
-        <v>159</v>
       </c>
       <c r="AG13" t="b">
         <v>0</v>
@@ -2696,16 +2693,16 @@
         <v>29</v>
       </c>
       <c r="B1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1" t="s">
         <v>160</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>161</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>162</v>
-      </c>
-      <c r="E1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2713,13 +2710,13 @@
         <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -2730,13 +2727,13 @@
         <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -2747,13 +2744,13 @@
         <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -2764,13 +2761,13 @@
         <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -2781,13 +2778,13 @@
         <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -2798,13 +2795,13 @@
         <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -2815,13 +2812,13 @@
         <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -2832,13 +2829,13 @@
         <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -2849,13 +2846,13 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -2866,13 +2863,13 @@
         <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -2883,13 +2880,13 @@
         <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C12" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -2900,13 +2897,13 @@
         <v>65</v>
       </c>
       <c r="B13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -2917,13 +2914,13 @@
         <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -2934,13 +2931,13 @@
         <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -2951,13 +2948,13 @@
         <v>66</v>
       </c>
       <c r="B16" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -2968,13 +2965,13 @@
         <v>66</v>
       </c>
       <c r="B17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -2985,13 +2982,13 @@
         <v>66</v>
       </c>
       <c r="B18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C18" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D18" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -3002,13 +2999,13 @@
         <v>67</v>
       </c>
       <c r="B19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D19" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -3019,13 +3016,13 @@
         <v>67</v>
       </c>
       <c r="B20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C20" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D20" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -3036,13 +3033,13 @@
         <v>67</v>
       </c>
       <c r="B21" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C21" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D21" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -3053,13 +3050,13 @@
         <v>68</v>
       </c>
       <c r="B22" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C22" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D22" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -3070,13 +3067,13 @@
         <v>68</v>
       </c>
       <c r="B23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C23" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -3087,13 +3084,13 @@
         <v>68</v>
       </c>
       <c r="B24" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C24" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -3104,13 +3101,13 @@
         <v>68</v>
       </c>
       <c r="B25" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C25" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D25" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -3121,13 +3118,13 @@
         <v>68</v>
       </c>
       <c r="B26" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C26" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D26" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -3138,13 +3135,13 @@
         <v>68</v>
       </c>
       <c r="B27" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D27" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -3155,13 +3152,13 @@
         <v>68</v>
       </c>
       <c r="B28" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C28" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D28" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -3172,13 +3169,13 @@
         <v>69</v>
       </c>
       <c r="B29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C29" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D29" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -3189,13 +3186,13 @@
         <v>69</v>
       </c>
       <c r="B30" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C30" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D30" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -3206,13 +3203,13 @@
         <v>69</v>
       </c>
       <c r="B31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C31" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D31" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -3223,13 +3220,13 @@
         <v>70</v>
       </c>
       <c r="B32" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C32" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D32" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -3240,13 +3237,13 @@
         <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D33" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -3257,13 +3254,13 @@
         <v>70</v>
       </c>
       <c r="B34" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C34" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D34" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -3274,13 +3271,13 @@
         <v>71</v>
       </c>
       <c r="B35" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C35" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D35" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -3291,13 +3288,13 @@
         <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D36" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -3308,13 +3305,13 @@
         <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C37" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -3325,13 +3322,13 @@
         <v>71</v>
       </c>
       <c r="B38" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D38" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -3345,10 +3342,10 @@
         <v>122</v>
       </c>
       <c r="C39" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D39" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -3372,16 +3369,16 @@
         <v>29</v>
       </c>
       <c r="B1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1" t="s">
         <v>204</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>205</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>206</v>
-      </c>
-      <c r="E1" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -3389,16 +3386,16 @@
         <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3406,16 +3403,16 @@
         <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3423,16 +3420,16 @@
         <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -3440,16 +3437,16 @@
         <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -3457,16 +3454,16 @@
         <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -3474,16 +3471,16 @@
         <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -3491,16 +3488,16 @@
         <v>64</v>
       </c>
       <c r="B8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -3508,16 +3505,16 @@
         <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D9" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -3525,16 +3522,16 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -3542,16 +3539,16 @@
         <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E11" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3559,16 +3556,16 @@
         <v>64</v>
       </c>
       <c r="B12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -3576,16 +3573,16 @@
         <v>65</v>
       </c>
       <c r="B13" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" t="s">
         <v>215</v>
       </c>
-      <c r="C13" t="s">
-        <v>216</v>
-      </c>
       <c r="D13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -3593,16 +3590,16 @@
         <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C14" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D14" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -3610,16 +3607,16 @@
         <v>65</v>
       </c>
       <c r="B15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -3627,16 +3624,16 @@
         <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C16" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D16" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E16" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -3644,16 +3641,16 @@
         <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D17" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E17" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -3661,16 +3658,16 @@
         <v>65</v>
       </c>
       <c r="B18" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C18" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E18" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -3678,16 +3675,16 @@
         <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C19" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -3695,16 +3692,16 @@
         <v>66</v>
       </c>
       <c r="B20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D20" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E20" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -3712,16 +3709,16 @@
         <v>66</v>
       </c>
       <c r="B21" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C21" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D21" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E21" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -3729,16 +3726,16 @@
         <v>66</v>
       </c>
       <c r="B22" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C22" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D22" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -3746,16 +3743,16 @@
         <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C23" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D23" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E23" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -3763,16 +3760,16 @@
         <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C24" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D24" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -3780,16 +3777,16 @@
         <v>67</v>
       </c>
       <c r="B25" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C25" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D25" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E25" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -3797,16 +3794,16 @@
         <v>67</v>
       </c>
       <c r="B26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C26" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D26" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E26" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -3814,16 +3811,16 @@
         <v>67</v>
       </c>
       <c r="B27" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C27" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E27" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -3831,16 +3828,16 @@
         <v>68</v>
       </c>
       <c r="B28" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C28" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D28" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E28" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -3848,16 +3845,16 @@
         <v>68</v>
       </c>
       <c r="B29" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C29" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D29" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E29" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -3865,16 +3862,16 @@
         <v>68</v>
       </c>
       <c r="B30" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C30" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D30" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E30" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -3882,16 +3879,16 @@
         <v>68</v>
       </c>
       <c r="B31" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C31" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D31" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -3899,16 +3896,16 @@
         <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D32" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E32" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -3916,16 +3913,16 @@
         <v>68</v>
       </c>
       <c r="B33" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C33" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D33" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E33" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -3933,16 +3930,16 @@
         <v>69</v>
       </c>
       <c r="B34" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C34" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D34" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E34" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -3950,16 +3947,16 @@
         <v>69</v>
       </c>
       <c r="B35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C35" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D35" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E35" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -3967,16 +3964,16 @@
         <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C36" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D36" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E36" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -3984,16 +3981,16 @@
         <v>69</v>
       </c>
       <c r="B37" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C37" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D37" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E37" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -4001,16 +3998,16 @@
         <v>70</v>
       </c>
       <c r="B38" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C38" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E38" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -4018,16 +4015,16 @@
         <v>70</v>
       </c>
       <c r="B39" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C39" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D39" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E39" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -4035,16 +4032,16 @@
         <v>70</v>
       </c>
       <c r="B40" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C40" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D40" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E40" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -4052,16 +4049,16 @@
         <v>70</v>
       </c>
       <c r="B41" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C41" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D41" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E41" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -4069,16 +4066,16 @@
         <v>71</v>
       </c>
       <c r="B42" t="s">
+        <v>214</v>
+      </c>
+      <c r="C42" t="s">
         <v>215</v>
       </c>
-      <c r="C42" t="s">
-        <v>216</v>
-      </c>
       <c r="D42" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E42" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -4086,16 +4083,16 @@
         <v>71</v>
       </c>
       <c r="B43" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C43" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D43" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E43" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -4103,16 +4100,16 @@
         <v>71</v>
       </c>
       <c r="B44" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C44" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D44" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E44" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -4120,16 +4117,16 @@
         <v>71</v>
       </c>
       <c r="B45" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C45" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D45" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E45" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -4137,16 +4134,16 @@
         <v>72</v>
       </c>
       <c r="B46" t="s">
+        <v>214</v>
+      </c>
+      <c r="C46" t="s">
         <v>215</v>
       </c>
-      <c r="C46" t="s">
-        <v>216</v>
-      </c>
       <c r="D46" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E46" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -4154,16 +4151,16 @@
         <v>72</v>
       </c>
       <c r="B47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C47" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D47" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E47" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -4171,16 +4168,16 @@
         <v>72</v>
       </c>
       <c r="B48" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C48" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D48" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E48" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -4188,16 +4185,16 @@
         <v>72</v>
       </c>
       <c r="B49" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C49" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D49" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E49" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -4205,16 +4202,16 @@
         <v>72</v>
       </c>
       <c r="B50" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C50" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D50" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E50" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -4222,16 +4219,16 @@
         <v>72</v>
       </c>
       <c r="B51" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C51" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D51" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E51" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -4239,16 +4236,16 @@
         <v>73</v>
       </c>
       <c r="B52" t="s">
+        <v>214</v>
+      </c>
+      <c r="C52" t="s">
         <v>215</v>
       </c>
-      <c r="C52" t="s">
-        <v>216</v>
-      </c>
       <c r="D52" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E52" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -4256,16 +4253,16 @@
         <v>73</v>
       </c>
       <c r="B53" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C53" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D53" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E53" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -4273,16 +4270,16 @@
         <v>73</v>
       </c>
       <c r="B54" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C54" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D54" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E54" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -4290,16 +4287,16 @@
         <v>73</v>
       </c>
       <c r="B55" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C55" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D55" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E55" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -4307,16 +4304,16 @@
         <v>73</v>
       </c>
       <c r="B56" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C56" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D56" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E56" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -4324,16 +4321,16 @@
         <v>74</v>
       </c>
       <c r="B57" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C57" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D57" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E57" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -4341,16 +4338,16 @@
         <v>74</v>
       </c>
       <c r="B58" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C58" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D58" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E58" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -4358,16 +4355,16 @@
         <v>74</v>
       </c>
       <c r="B59" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C59" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D59" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E59" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -4375,16 +4372,16 @@
         <v>74</v>
       </c>
       <c r="B60" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C60" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D60" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E60" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -4392,16 +4389,16 @@
         <v>74</v>
       </c>
       <c r="B61" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C61" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D61" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E61" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -4419,37 +4416,37 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B1" t="s">
         <v>30</v>
       </c>
       <c r="C1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D1" t="s">
         <v>32</v>
       </c>
       <c r="E1" t="s">
+        <v>297</v>
+      </c>
+      <c r="F1" t="s">
         <v>298</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>299</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>300</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>301</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>302</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>303</v>
-      </c>
-      <c r="K1" t="s">
-        <v>304</v>
       </c>
       <c r="L1" t="s">
         <v>48</v>
@@ -4457,13 +4454,13 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B2" t="s">
         <v>77</v>
       </c>
       <c r="C2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D2" t="s">
         <v>82</v>
@@ -4472,36 +4469,36 @@
         <v>85</v>
       </c>
       <c r="F2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I2" t="b">
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="K2" t="s">
+        <v>323</v>
+      </c>
+      <c r="L2" t="s">
         <v>324</v>
-      </c>
-      <c r="L2" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B3" t="s">
         <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D3" t="s">
         <v>82</v>
@@ -4510,36 +4507,36 @@
         <v>89</v>
       </c>
       <c r="F3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I3" t="b">
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="K3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="L3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B4" t="s">
         <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D4" t="s">
         <v>82</v>
@@ -4548,36 +4545,36 @@
         <v>86</v>
       </c>
       <c r="F4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I4" t="b">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="K4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="L4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B5" t="s">
         <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D5" t="s">
         <v>81</v>
@@ -4586,25 +4583,25 @@
         <v>93</v>
       </c>
       <c r="F5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G5" t="s">
+        <v>318</v>
+      </c>
+      <c r="H5" t="s">
+        <v>321</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="s">
         <v>319</v>
       </c>
-      <c r="H5" t="s">
-        <v>322</v>
-      </c>
-      <c r="I5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
-        <v>320</v>
-      </c>
       <c r="K5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="L5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -4622,12 +4619,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -4645,12 +4642,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>